<commit_message>
test(seguridad): PS-01c aprobada en produccion (HU-17, 3/3)
</commit_message>
<xml_diff>
--- a/docs/fase2/evidencias_proyecto/documentacion/trazabilidad.xlsx
+++ b/docs/fase2/evidencias_proyecto/documentacion/trazabilidad.xlsx
@@ -1580,7 +1580,7 @@
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Solo el cuidador autenticado puede atender alertas</t>
+          <t>Solo el cuidador autenticado puede atender alertas y consultar los datos del hogar</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
@@ -1595,17 +1595,17 @@
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>backend/auth_cuidador.py; Supabase Auth</t>
+          <t>backend/auth_cuidador.py; Supabase Auth; verificar_lectura (HU-17)</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>PS-01b</t>
+          <t>PS-01b, PS-01c</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
         <is>
-          <t>3/3 en producción</t>
+          <t>3/3 en producción (atender alertas) y 3/3 en producción (consultas de lectura con PROTEGER_LECTURAS=1)</t>
         </is>
       </c>
       <c r="I22" s="23" t="inlineStr">

</xml_diff>

<commit_message>
feat(borde): PR-03b aprobada (5/5 sincronizadas), hora real en avisos tardios, documentacion HU-03
</commit_message>
<xml_diff>
--- a/docs/fase2/evidencias_proyecto/documentacion/trazabilidad.xlsx
+++ b/docs/fase2/evidencias_proyecto/documentacion/trazabilidad.xlsx
@@ -815,17 +815,17 @@
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>backend/database.py (SQLite, modo borde)</t>
+          <t>backend/database.py (SQLite, modo borde); backend/sincronizador.py (HU-03)</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
         <is>
-          <t>PR-03</t>
+          <t>PR-03, PU-07, PR-03b</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>10/10 caídas guardadas y mostradas sin internet; sin sincronización automática</t>
+          <t>10/10 caídas sin internet (PR-03); al volver la conexión, 5/5 sincronizadas con Supabase sin duplicados (PR-03b); PU-07 13/13</t>
         </is>
       </c>
       <c r="I7" s="23" t="inlineStr">
@@ -833,9 +833,9 @@
           <t>docs/fase2/evidencias_proyecto/documentacion/capturas/PR-03_consola_10de10_sin_internet.png; docs/fase2/evidencias_proyecto/documentacion/capturas/PR-03_sqlite_30_eventos.png</t>
         </is>
       </c>
-      <c r="J7" s="25" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+      <c r="J7" s="24" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
         </is>
       </c>
     </row>
@@ -1699,17 +1699,17 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>SQLite local; panel local</t>
+          <t>SQLite local; panel local; backend/sincronizador.py (HU-03)</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>PR-03</t>
+          <t>PR-03, PU-07, PR-03b</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
         <is>
-          <t>10/10 sin internet; falta sincronización al reconectar</t>
+          <t>10/10 caídas sin internet (PR-03); al volver la conexión, 5/5 sincronizadas con Supabase sin duplicados (PR-03b); PU-07 13/13</t>
         </is>
       </c>
       <c r="I24" s="23" t="inlineStr">
@@ -1717,9 +1717,9 @@
           <t>docs/fase2/evidencias_proyecto/documentacion/capturas/PR-03_panel_local_sin_internet_ntfy_offline.png</t>
         </is>
       </c>
-      <c r="J24" s="25" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+      <c r="J24" s="24" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
         </is>
       </c>
     </row>

</xml_diff>